<commit_message>
Switch Powder Room 2 to Top Knobs Emerald pull; add PDF of 10C hardware sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NPYSfnsS6GJpbxy7jbeH4k
</commit_message>
<xml_diff>
--- a/docs/10C-Hardware.xlsx
+++ b/docs/10C-Hardware.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="44">
   <si>
     <t xml:space="preserve">10C Hardware Selections</t>
   </si>
@@ -149,10 +149,10 @@
     <t xml:space="preserve">Powder Room 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Liberty Hardware</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chamfered Slim Bar Pull</t>
+    <t xml:space="preserve">Emerald Pull</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finish matches Bathroom 1 / Powder Room 1; size preselected in link – confirm with Rich</t>
   </si>
   <si>
     <t xml:space="preserve">Master Bath</t>
@@ -668,7 +668,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:L13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -901,7 +901,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
         <v>33</v>
       </c>
@@ -909,13 +909,13 @@
         <v>15</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>35</v>
-      </c>
       <c r="E10" s="4" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>19</v>
@@ -932,7 +932,9 @@
       <c r="K10" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="L10" s="4"/>
+      <c r="L10" s="4" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
@@ -1029,8 +1031,8 @@
     <hyperlink ref="J11" r:id="rId8" display="View product"/>
     <hyperlink ref="J12" r:id="rId9" display="View product"/>
   </hyperlinks>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
+  <pageMargins left="0.4" right="0.4" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>

</xml_diff>

<commit_message>
Add finishes to 10C hardware sheet; switch PDF to portrait
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NPYSfnsS6GJpbxy7jbeH4k
</commit_message>
<xml_diff>
--- a/docs/10C-Hardware.xlsx
+++ b/docs/10C-Hardware.xlsx
@@ -11,7 +11,7 @@
     <sheet name="10C Hardware" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'10C Hardware'!$A$4:$L$12</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'10C Hardware'!$A$4:$K$12</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -28,7 +28,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="F4" authorId="0">
+    <comment ref="E4" authorId="0">
       <text>
         <r>
           <rPr>
@@ -45,9 +45,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="44">
-  <si>
-    <t xml:space="preserve">10C Hardware Selections</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="42">
+  <si>
+    <t xml:space="preserve">10C Hardware Selections – Cabinet Pulls</t>
   </si>
   <si>
     <t xml:space="preserve">Sizing to be determined by Rich. Yellow cells are to be filled in; Total and Grand Total calculate automatically.</t>
@@ -56,9 +56,6 @@
     <t xml:space="preserve">Room</t>
   </si>
   <si>
-    <t xml:space="preserve">Item</t>
-  </si>
-  <si>
     <t xml:space="preserve">Brand</t>
   </si>
   <si>
@@ -92,16 +89,13 @@
     <t xml:space="preserve">Bathroom 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Cabinet Pulls</t>
-  </si>
-  <si>
     <t xml:space="preserve">Top Knobs</t>
   </si>
   <si>
     <t xml:space="preserve">Riverside Pull</t>
   </si>
   <si>
-    <t xml:space="preserve">Per link (finish preselected)</t>
+    <t xml:space="preserve">Honey Bronze</t>
   </si>
   <si>
     <t xml:space="preserve">TBD – Rich</t>
@@ -119,7 +113,7 @@
     <t xml:space="preserve">Morris Pull</t>
   </si>
   <si>
-    <t xml:space="preserve">TBD</t>
+    <t xml:space="preserve">Brushed Nickel</t>
   </si>
   <si>
     <t xml:space="preserve">Bathroom 3</t>
@@ -128,6 +122,9 @@
     <t xml:space="preserve">Lydia Pull</t>
   </si>
   <si>
+    <t xml:space="preserve">Chrome</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bathroom 5</t>
   </si>
   <si>
@@ -137,7 +134,7 @@
     <t xml:space="preserve">Parow Pull</t>
   </si>
   <si>
-    <t xml:space="preserve">Per link (variant preselected)</t>
+    <t xml:space="preserve">Black</t>
   </si>
   <si>
     <t xml:space="preserve">Powder Room 1</t>
@@ -152,7 +149,7 @@
     <t xml:space="preserve">Emerald Pull</t>
   </si>
   <si>
-    <t xml:space="preserve">Finish matches Bathroom 1 / Powder Room 1; size preselected in link – confirm with Rich</t>
+    <t xml:space="preserve">Size preselected in link – confirm with Rich</t>
   </si>
   <si>
     <t xml:space="preserve">Master Bath</t>
@@ -164,10 +161,7 @@
     <t xml:space="preserve">Pull, 5-1/16" (128mm) centers – BP36655CCZ</t>
   </si>
   <si>
-    <t xml:space="preserve">Clear &amp; Champagne Bronze</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inspiration only – "something like this"</t>
+    <t xml:space="preserve">Inspiration only – "something like this"; linked example is Champagne Bronze, selection is Honey Bronze</t>
   </si>
   <si>
     <t xml:space="preserve">Kitchen</t>
@@ -670,20 +664,20 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -696,7 +690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -730,115 +724,103 @@
       <c r="K4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="L4" s="3" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="5"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="7" t="str">
+        <f aca="false">IF(OR(F5="",G5=""),"",F5*G5)</f>
+        <v/>
+      </c>
+      <c r="I5" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="J5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="5"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="7" t="str">
-        <f aca="false">IF(OR(G5="",H5=""),"",G5*H5)</f>
-        <v/>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="L5" s="4"/>
+      <c r="K5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>23</v>
-      </c>
       <c r="E6" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="5"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="7" t="str">
+        <f aca="false">IF(OR(F6="",G6=""),"",F6*G6)</f>
+        <v/>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G6" s="5"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="7" t="str">
-        <f aca="false">IF(OR(G6="",H6=""),"",G6*H6)</f>
-        <v/>
-      </c>
-      <c r="J6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="L6" s="4"/>
+      <c r="K6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>26</v>
-      </c>
       <c r="E7" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="5"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="7" t="str">
+        <f aca="false">IF(OR(F7="",G7=""),"",F7*G7)</f>
+        <v/>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G7" s="5"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="7" t="str">
-        <f aca="false">IF(OR(G7="",H7=""),"",G7*H7)</f>
-        <v/>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="L7" s="4"/>
+      <c r="K7" s="4"/>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>15</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>28</v>
@@ -846,194 +828,179 @@
       <c r="D8" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F8" s="5" t="s">
+      <c r="E8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="5"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="7" t="str">
+        <f aca="false">IF(OR(F8="",G8=""),"",F8*G8)</f>
+        <v/>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="5"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="7" t="str">
-        <f aca="false">IF(OR(G8="",H8=""),"",G8*H8)</f>
-        <v/>
-      </c>
-      <c r="J8" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="L8" s="4"/>
+      <c r="K8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="5"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="7" t="str">
+        <f aca="false">IF(OR(F9="",G9=""),"",F9*G9)</f>
+        <v/>
+      </c>
+      <c r="I9" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K9" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="4" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E9" s="4" t="s">
+      <c r="E10" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" s="5"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="7" t="str">
+        <f aca="false">IF(OR(F10="",G10=""),"",F10*G10)</f>
+        <v/>
+      </c>
+      <c r="I10" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="J10" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G9" s="5"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="7" t="str">
-        <f aca="false">IF(OR(G9="",H9=""),"",G9*H9)</f>
-        <v/>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="L9" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D10" s="4" t="s">
+      <c r="K10" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G10" s="5"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="7" t="str">
-        <f aca="false">IF(OR(G10="",H10=""),"",G10*H10)</f>
-        <v/>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="L10" s="4" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="B11" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>15</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>37</v>
       </c>
       <c r="D11" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" s="5"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="7" t="str">
+        <f aca="false">IF(OR(F11="",G11=""),"",F11*G11)</f>
+        <v/>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K11" s="4" t="s">
         <v>38</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G11" s="5"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="7" t="str">
-        <f aca="false">IF(OR(G11="",H11=""),"",G11*H11)</f>
-        <v/>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="L11" s="4" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" s="5"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="7" t="str">
+        <f aca="false">IF(OR(F12="",G12=""),"",F12*G12)</f>
+        <v/>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K12" s="4"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G13" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G12" s="5"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="7" t="str">
-        <f aca="false">IF(OR(G12="",H12=""),"",G12*H12)</f>
-        <v/>
-      </c>
-      <c r="J12" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="L12" s="4"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H13" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="I13" s="10" t="n">
-        <f aca="false">SUM(I5:I12)</f>
+      <c r="H13" s="10" t="n">
+        <f aca="false">SUM(H5:H12)</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L12"/>
+  <autoFilter ref="A4:K12"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K5:K12" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J12" type="list">
       <formula1>"Pending,Approved,Ordered,Received,Installed"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="J5" r:id="rId2" display="View product"/>
-    <hyperlink ref="J6" r:id="rId3" display="View product"/>
-    <hyperlink ref="J7" r:id="rId4" display="View product"/>
-    <hyperlink ref="J8" r:id="rId5" display="View product"/>
-    <hyperlink ref="J9" r:id="rId6" display="View product"/>
-    <hyperlink ref="J10" r:id="rId7" display="View product"/>
-    <hyperlink ref="J11" r:id="rId8" display="View product"/>
-    <hyperlink ref="J12" r:id="rId9" display="View product"/>
+    <hyperlink ref="I5" r:id="rId2" display="View product"/>
+    <hyperlink ref="I6" r:id="rId3" display="View product"/>
+    <hyperlink ref="I7" r:id="rId4" display="View product"/>
+    <hyperlink ref="I8" r:id="rId5" display="View product"/>
+    <hyperlink ref="I9" r:id="rId6" display="View product"/>
+    <hyperlink ref="I10" r:id="rId7" display="View product"/>
+    <hyperlink ref="I11" r:id="rId8" display="View product"/>
+    <hyperlink ref="I12" r:id="rId9" display="View product"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
   <pageMargins left="0.4" right="0.4" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>